<commit_message>
Add AIiH (International Conference on AI in Healthcare) 2027
User-requested addition reviewed from the official site (aiih.cc) on
2026-10-29: fourth edition at the Mathematical Institute, University of
Oxford, Sep 1-3, 2027.

- Independent full-paper and abstract routes due Apr 9, 2027 and a
  late-breaking abstract/STARS survey route due Jul 2. The site states
  "11.59PM Pacific Time (GMT-8)"; -08:00 is stored as published and the
  notes flag that Pacific clocks are on GMT-7 then.
- Healthcare central identity, curated scope profile, Oxford map alias and
  annual rollover cadence (editions 2024-2027). No ICORE/CCF rank mapped.
- Workbook catalog and scope tables extended by one row each; addition
  regression tests; payload-count test now derives counts from data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N130" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -151,7 +151,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Series"/>
     <x:tableColumn id="2" name="Additional topics"/>
@@ -4737,6 +4737,34 @@
       <x:c r="M130"/>
       <x:c r="N130"/>
     </x:row>
+    <x:row r="131" ht="15" hidden="0" customHeight="1">
+      <x:c r="A131" t="str">
+        <x:v>AIiH</x:v>
+      </x:c>
+      <x:c r="B131" s="12" t="str">
+        <x:v>Healthcare &amp; Clinical AI; Biomedical Imaging; Machine Learning; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E131"/>
+      <x:c r="F131" s="12" t="str">
+        <x:v>Full papers (double-blind, proceedings) or abstracts (posters/spotlights, Zenodo); late-breaking abstracts and STARS surveys</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>https://aiih.cc/</x:v>
+      </x:c>
+      <x:c r="H131"/>
+      <x:c r="I131"/>
+      <x:c r="J131"/>
+      <x:c r="K131" s="16"/>
+      <x:c r="L131" s="17"/>
+      <x:c r="M131"/>
+      <x:c r="N131"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
@@ -6713,6 +6741,26 @@
         <x:v>46302</x:v>
       </x:c>
     </x:row>
+    <x:row r="81" ht="60" hidden="0" customHeight="1">
+      <x:c r="A81" s="20" t="str">
+        <x:v>AIiH</x:v>
+      </x:c>
+      <x:c r="B81" s="20" t="str">
+        <x:v>Ethics &amp; Governance; Privacy-preserving ML; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C81" s="20" t="str">
+        <x:v>Artificial intelligence for healthcare and medicine, including predictive analytics, early diagnosis and prevention, machine and deep learning on health data, AI-aided medical signal processing and imaging, digital pathology and neurology, drug discovery, digital twins and precision medicine. Ethics, patient data privacy and patient-centred deployment are recurring themes. Original research papers, abstracts and state-of-the-art surveys are accepted.</x:v>
+      </x:c>
+      <x:c r="D81" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E81" s="20" t="str">
+        <x:v>https://aiih.cc/call-for-papers/; https://aiih.cc/call-for-stars/</x:v>
+      </x:c>
+      <x:c r="F81" s="22" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">

</xml_diff>

<commit_message>
Apply owner decisions: earliest conflicting cutoffs, SD4H as TS4H successor, ISBI extension
- Conflicting official cutoffs store the earliest stated instant with a
  cutoff_note: IEEE BHI 2026 late abstracts, MLSys 2027 (noon PDT; opening
  now Oct 19 20:00 UTC), IDA 2027, AIS 2027 regular papers, AIiH 2027 and
  ACC 2028. These records were re-read on 2026-10-29.
- Track Structured Data for Health (SD4H 2026, ICML 2026) as TS4H's
  successor under the TS4H series key; the workbook's TS4H row follows it.
- ISBI 2027 paper deadline extended to Nov 2, 2026, 11:59 pm ET.
- ICPRv is not tracked and the ICCN 2026 record is kept (no data change).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -920,7 +920,7 @@
         <x:v>TS4H</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI; Signal Processing; Explainability &amp; Interpretability</x:v>
+        <x:v>Healthcare &amp; Clinical AI; Time Series &amp; Sequential Data; Signal Processing; Deep Representation Learning</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
         <x:v>S</x:v>
@@ -930,10 +930,10 @@
       </x:c>
       <x:c r="E16" s="14"/>
       <x:c r="F16" s="14" t="str">
-        <x:v>Workshop / paper-based</x:v>
+        <x:v>Workshop / non-archival short paper</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>https://timeseries4health.github.io/</x:v>
+        <x:v>https://structureddata4health.github.io/</x:v>
       </x:c>
       <x:c r="H16"/>
       <x:c r="I16"/>

</xml_diff>